<commit_message>
Expand nine-package decision support analysis
</commit_message>
<xml_diff>
--- a/demo_data/synthetic/P01_Store_Sales_Inventory_SYNTHETIC.xlsx
+++ b/demo_data/synthetic/P01_Store_Sales_Inventory_SYNTHETIC.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9163801f179e49fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1033a03deb904c99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,11 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="#,##0"/>
-    <x:numFmt numFmtId="201" formatCode="0.0%"/>
-  </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -28,14 +24,8 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF6F4B00"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -44,89 +34,139 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF174F3B"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF0C9"/>
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="10">
     <x:border/>
     <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:right>
       <x:bottom style="thin">
-        <x:color rgb="FFE0E3DE"/>
+        <x:color rgb="FFD9E0DC"/>
       </x:bottom>
     </x:border>
     <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:right>
       <x:top style="thin">
-        <x:color rgb="FFE0E3DE"/>
+        <x:color rgb="FFD9E0DC"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFE0E3DE"/>
+        <x:color rgb="FFD9E0DC"/>
       </x:bottom>
     </x:border>
     <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:right>
       <x:top style="thin">
-        <x:color rgb="FFE0E3DE"/>
+        <x:color rgb="FFD9E0DC"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFC8CDC7"/>
+        <x:color rgb="FFD9E0DC"/>
       </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E0DC"/>
+      </x:top>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_P01StoreSalesInvento" displayName="T_P01StoreSalesInvento" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="11">
-    <x:tableColumn id="1" name="walmart_calendar_week"/>
-    <x:tableColumn id="2" name="vendor_stock_id"/>
-    <x:tableColumn id="3" name="walmart_item_number"/>
-    <x:tableColumn id="4" name="item_name"/>
-    <x:tableColumn id="5" name="store_number"/>
-    <x:tableColumn id="6" name="pos_quantity_this_year"/>
-    <x:tableColumn id="7" name="pos_sales_this_year"/>
-    <x:tableColumn id="8" name="store_on_hand_quantity_this_year"/>
-    <x:tableColumn id="9" name="store_on_order_quantity_this_year"/>
-    <x:tableColumn id="10" name="repl_instock_percentage_this_year"/>
-    <x:tableColumn id="11" name="data_classification"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -324,21 +364,22 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="52" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="34" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="5" t="str">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="4" t="str">
         <x:v>walmart_calendar_week</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
@@ -369,118 +410,127 @@
         <x:v>repl_instock_percentage_this_year</x:v>
       </x:c>
       <x:c r="K1" s="5" t="str">
+        <x:v>actual_order_quantity_last_4_weeks</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
         <x:v>data_classification</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="6" t="str">
+    <x:row r="2" ht="42" hidden="0" customHeight="1">
+      <x:c r="A2" s="7" t="str">
         <x:v>202630</x:v>
       </x:c>
-      <x:c r="B2" s="6" t="str">
+      <x:c r="B2" s="8" t="str">
         <x:v>DEMO-SURPLUS</x:v>
       </x:c>
-      <x:c r="C2" s="6" t="str">
+      <x:c r="C2" s="8" t="str">
         <x:v>900000001</x:v>
       </x:c>
-      <x:c r="D2" s="6" t="str">
+      <x:c r="D2" s="8" t="str">
         <x:v>Synthetic Comfort Wrap</x:v>
       </x:c>
-      <x:c r="E2" s="6" t="str">
+      <x:c r="E2" s="8" t="str">
         <x:v>0101</x:v>
       </x:c>
-      <x:c r="F2" s="12" t="n">
+      <x:c r="F2" s="8" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="G2" s="6" t="n">
+      <x:c r="G2" s="8" t="n">
         <x:v>2398.8</x:v>
       </x:c>
-      <x:c r="H2" s="12" t="n">
+      <x:c r="H2" s="8" t="n">
         <x:v>420</x:v>
       </x:c>
-      <x:c r="I2" s="12" t="n">
+      <x:c r="I2" s="8" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="J2" s="14" t="n">
+      <x:c r="J2" s="8" t="n">
         <x:v>0.96</x:v>
       </x:c>
-      <x:c r="K2" s="10" t="str">
+      <x:c r="K2" s="8" t="n">
+        <x:v>2200</x:v>
+      </x:c>
+      <x:c r="L2" s="13" t="str">
         <x:v>SYNTHETIC DEMONSTRATION DATA - NOT FOR OPERATIONAL USE</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="6" t="str">
+    <x:row r="3" ht="42" hidden="0" customHeight="1">
+      <x:c r="A3" s="7" t="str">
         <x:v>202630</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="8" t="str">
         <x:v>DEMO-SHORTAGE</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="8" t="str">
         <x:v>900000002</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="8" t="str">
         <x:v>Synthetic Cooling Patch</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="8" t="str">
         <x:v>0101</x:v>
       </x:c>
-      <x:c r="F3" s="12" t="n">
+      <x:c r="F3" s="8" t="n">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="G3" s="6" t="n">
+      <x:c r="G3" s="8" t="n">
         <x:v>2698.2</x:v>
       </x:c>
-      <x:c r="H3" s="12" t="n">
+      <x:c r="H3" s="8" t="n">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="I3" s="12" t="n">
+      <x:c r="I3" s="8" t="n">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="J3" s="14" t="n">
+      <x:c r="J3" s="8" t="n">
         <x:v>0.84</x:v>
       </x:c>
-      <x:c r="K3" s="10" t="str">
+      <x:c r="K3" s="8" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="L3" s="13" t="str">
         <x:v>SYNTHETIC DEMONSTRATION DATA - NOT FOR OPERATIONAL USE</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="7" t="str">
+    <x:row r="4" ht="42" hidden="0" customHeight="1">
+      <x:c r="A4" s="10" t="str">
         <x:v>202630</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>DEMO-LATE</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="str">
+      <x:c r="C4" s="11" t="str">
         <x:v>900000003</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="str">
+      <x:c r="D4" s="11" t="str">
         <x:v>Synthetic Travel Cushion</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="str">
+      <x:c r="E4" s="11" t="str">
         <x:v>0101</x:v>
       </x:c>
-      <x:c r="F4" s="13" t="n">
+      <x:c r="F4" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="G4" s="7" t="n">
+      <x:c r="G4" s="11" t="n">
         <x:v>3599.1</x:v>
       </x:c>
-      <x:c r="H4" s="13" t="n">
+      <x:c r="H4" s="11" t="n">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="I4" s="13" t="n">
+      <x:c r="I4" s="11" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="J4" s="15" t="n">
+      <x:c r="J4" s="11" t="n">
         <x:v>0.89</x:v>
       </x:c>
-      <x:c r="K4" s="11" t="str">
+      <x:c r="K4" s="11" t="n">
+        <x:v>1960</x:v>
+      </x:c>
+      <x:c r="L4" s="14" t="str">
         <x:v>SYNTHETIC DEMONSTRATION DATA - NOT FOR OPERATIONAL USE</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R972f074d9b924188"/>
-  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>